<commit_message>
Update guidelines for R programming: add usage of 'fs' for file system operations and clarify 'future' for parallel computing.
</commit_message>
<xml_diff>
--- a/templates/Nomeador de arquivos.xlsx
+++ b/templates/Nomeador de arquivos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://incorporadoraampla.sharepoint.com/sites/Controladoria/Documentos Compartilhados/amplaGitHub/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="199" documentId="11_8BDB85793461764BD106A2AB1F101464FD041DB6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{06A59B93-7E2B-46C7-A950-6861F560C2B4}"/>
+  <xr:revisionPtr revIDLastSave="207" documentId="11_8BDB85793461764BD106A2AB1F101464FD041DB6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E3E0B37-CCC6-4E7A-8FBA-0837DB6F4D2E}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1305" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>Tipos de arquivo</t>
   </si>
@@ -126,9 +126,6 @@
   </si>
   <si>
     <t>O nome do arquivo deve ser:</t>
-  </si>
-  <si>
-    <t>Julho</t>
   </si>
   <si>
     <t>Basta preencher as 4 células com bordas vermelhas e copiar o nome do arquivo!</t>
@@ -265,7 +262,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -636,7 +633,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:J50"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" zeroHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.7109375" customWidth="1"/>
@@ -646,15 +643,15 @@
     <col min="5" max="5" width="20.7109375" customWidth="1"/>
     <col min="6" max="6" width="38" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="3.7109375" customWidth="1"/>
-    <col min="8" max="8" width="33.7109375" hidden="1"/>
-    <col min="9" max="9" width="9.140625" hidden="1"/>
-    <col min="10" max="10" width="20.7109375" hidden="1"/>
+    <col min="8" max="8" width="33.7109375" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="9.140625" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="20.7109375" hidden="1" customWidth="1"/>
     <col min="11" max="16384" width="9.140625" hidden="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B1" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="2:6" x14ac:dyDescent="0.25"/>
@@ -663,29 +660,23 @@
         <v>27</v>
       </c>
       <c r="C3" s="3"/>
-      <c r="D3" s="6" t="s">
-        <v>26</v>
-      </c>
+      <c r="D3" s="6"/>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25"/>
     <row r="5" spans="2:6" ht="21" x14ac:dyDescent="0.35">
       <c r="B5" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" s="6">
-        <v>2025</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>30</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
       <c r="F5" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="F6" s="2" t="str">
+      <c r="F6" s="2" t="e">
         <f>_xlfn.CONCAT(IF(D3="Contratos (contr)","Contratos",IF(D3="Inadimplencia (inad)","Inadimplencia","")),"-",D7,"-",C5,"_",_xlfn.IFS(D5="Janeiro","01",D5="Fevereiro","02",D5="Março","03",D5="Abril","04",D5="Maio","05",D5="Junho","06",D5="Julho","07",D5="Agosto","08",D5="Setembro","09",D5="Outubro",10,D5="Novembro","11",D5="Dezembro","12"))</f>
-        <v>Contratos-AVS-2025_07</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="7" spans="2:6" ht="21" x14ac:dyDescent="0.35">
@@ -693,9 +684,7 @@
         <v>28</v>
       </c>
       <c r="C7" s="3"/>
-      <c r="D7" s="6" t="s">
-        <v>3</v>
-      </c>
+      <c r="D7" s="6"/>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25"/>
     <row r="9" spans="2:6" x14ac:dyDescent="0.25"/>
@@ -856,7 +845,7 @@
       <formula>LEN(TRIM(C3))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations disablePrompts="1" count="4">
+  <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3" xr:uid="{6DF6D08E-F022-470A-82EF-7926C5CC47C9}">
       <formula1>INDIRECT("tipos[Tipos de arquivo]")</formula1>
     </dataValidation>
@@ -891,6 +880,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006C56FB2846673243A9735D5EC6051572" ma:contentTypeVersion="11" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="36569ac63cfce8ff0f8884bc80e67f1c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5a5f483f-f768-438e-b4ef-63f46a7558dd" xmlns:ns3="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2040da04b75a9ea4fe796fa8180f8ca6" ns2:_="" ns3:_="">
     <xsd:import namespace="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
@@ -1085,15 +1083,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{637A4E3A-2793-49F4-B2B5-E8D79756ECAC}">
   <ds:schemaRefs>
@@ -1106,6 +1095,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{380F78C4-C2DB-4920-B426-698322055391}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E5D4FB3-33A8-4BDC-8357-D4F39476A52A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1122,12 +1119,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{380F78C4-C2DB-4920-B426-698322055391}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Refactor caminhos_pastas function to enhance path management; streamline project paths using here() for portability and remove redundant definitions.
</commit_message>
<xml_diff>
--- a/templates/Nomeador de arquivos.xlsx
+++ b/templates/Nomeador de arquivos.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29101"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://incorporadoraampla.sharepoint.com/sites/Controladoria/Documentos Compartilhados/amplaGitHub/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="207" documentId="11_8BDB85793461764BD106A2AB1F101464FD041DB6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E3E0B37-CCC6-4E7A-8FBA-0837DB6F4D2E}"/>
+  <xr:revisionPtr revIDLastSave="211" documentId="11_8BDB85793461764BD106A2AB1F101464FD041DB6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E1B558C-7DB6-4C72-878C-BA66BE5A1C3F}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1305" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nomeador" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,31 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
+  <si>
+    <t>Basta preencher as 4 células com bordas vermelhas e copiar o nome do arquivo!</t>
+  </si>
+  <si>
+    <t>1. Qual é o tipo do arquivo a ser nomeado?</t>
+  </si>
+  <si>
+    <t>Contratos (contr)</t>
+  </si>
+  <si>
+    <t>2. Qual é o ano e o mês de referência do arquivo?</t>
+  </si>
+  <si>
+    <t>Julho</t>
+  </si>
+  <si>
+    <t>O nome do arquivo deve ser:</t>
+  </si>
+  <si>
+    <t>3. O arquivo se refere a qual empreendimento?</t>
+  </si>
+  <si>
+    <t>BUT</t>
+  </si>
   <si>
     <t>Tipos de arquivo</t>
   </si>
@@ -47,12 +71,12 @@
     <t>AVR</t>
   </si>
   <si>
+    <t>Inadimplencia (inad)</t>
+  </si>
+  <si>
     <t>AVS</t>
   </si>
   <si>
-    <t>BUT</t>
-  </si>
-  <si>
     <t>CBL</t>
   </si>
   <si>
@@ -111,34 +135,13 @@
   </si>
   <si>
     <t>USL</t>
-  </si>
-  <si>
-    <t>Inadimplencia (inad)</t>
-  </si>
-  <si>
-    <t>Contratos (contr)</t>
-  </si>
-  <si>
-    <t>1. Qual é o tipo do arquivo a ser nomeado?</t>
-  </si>
-  <si>
-    <t>3. O arquivo se refere a qual empreendimento?</t>
-  </si>
-  <si>
-    <t>O nome do arquivo deve ser:</t>
-  </si>
-  <si>
-    <t>Basta preencher as 4 células com bordas vermelhas e copiar o nome do arquivo!</t>
-  </si>
-  <si>
-    <t>2. Qual é o ano e o mês de referência do arquivo?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -272,17 +275,17 @@
   </cellStyles>
   <dxfs count="3">
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -362,9 +365,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0B4EABC4-6A33-4718-9BCE-E1A3BA547DAE}" name="empreendimentos" displayName="empreendimentos" ref="E11:E34" totalsRowShown="0" dataDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0B4EABC4-6A33-4718-9BCE-E1A3BA547DAE}" name="empreendimentos" displayName="empreendimentos" ref="E11:E34" totalsRowShown="0" dataDxfId="1">
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{9FD3D6E2-4108-48F3-8813-131FF4BB2FC6}" name="Empreendimentos" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{9FD3D6E2-4108-48F3-8813-131FF4BB2FC6}" name="Empreendimentos" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -634,7 +637,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J50"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" zeroHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" zeroHeight="1"/>
   <cols>
     <col min="1" max="1" width="3.7109375" customWidth="1"/>
     <col min="2" max="2" width="64.85546875" bestFit="1" customWidth="1"/>
@@ -649,191 +652,199 @@
     <col min="11" max="16384" width="9.140625" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:6">
       <c r="B1" s="7" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="2:6"/>
+    <row r="3" spans="2:6" ht="21">
+      <c r="B3" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="3"/>
+      <c r="D3" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6"/>
+    <row r="5" spans="2:6" ht="21">
+      <c r="B5" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="6">
+        <v>2025</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6">
+      <c r="F6" s="2" t="str">
+        <f>_xlfn.CONCAT(IF(D3="Contratos (contr)","Contratos",IF(D3="Inadimplencia (inad)","Inadimplencia","")),"-",D7,"-",C5,"_",_xlfn.IFS(D5="Janeiro","01",D5="Fevereiro","02",D5="Março","03",D5="Abril","04",D5="Maio","05",D5="Junho","06",D5="Julho","07",D5="Agosto","08",D5="Setembro","09",D5="Outubro",10,D5="Novembro","11",D5="Dezembro","12"))</f>
+        <v>Contratos-BUT-2025_07</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" ht="21">
+      <c r="B7" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="3"/>
+      <c r="D7" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6"/>
+    <row r="9" spans="2:6"/>
+    <row r="10" spans="2:6"/>
+    <row r="11" spans="2:6">
+      <c r="B11" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6">
+      <c r="B12" t="s">
+        <v>2</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6">
+      <c r="B13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6">
+      <c r="E14" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6">
+      <c r="E15" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6">
+      <c r="E16" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="5:5">
+      <c r="E17" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="5:5">
+      <c r="E18" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="5:5">
+      <c r="E19" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="5:5">
+      <c r="E20" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="5:5">
+      <c r="E21" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="5:5">
+      <c r="E22" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="5:5">
+      <c r="E23" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="5:5">
+      <c r="E24" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" spans="5:5">
+      <c r="E25" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="26" spans="5:5">
+      <c r="E26" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="5:5">
+      <c r="E27" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="28" spans="5:5">
+      <c r="E28" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="5:5">
+      <c r="E29" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30" spans="5:5">
+      <c r="E30" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="31" spans="5:5">
+      <c r="E31" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="32" spans="5:5">
+      <c r="E32" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="2:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="B3" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="6"/>
-    </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="2:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="B5" s="5" t="s">
+    <row r="33" spans="5:5">
+      <c r="E33" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="F5" s="4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="F6" s="2" t="e">
-        <f>_xlfn.CONCAT(IF(D3="Contratos (contr)","Contratos",IF(D3="Inadimplencia (inad)","Inadimplencia","")),"-",D7,"-",C5,"_",_xlfn.IFS(D5="Janeiro","01",D5="Fevereiro","02",D5="Março","03",D5="Abril","04",D5="Maio","05",D5="Junho","06",D5="Julho","07",D5="Agosto","08",D5="Setembro","09",D5="Outubro",10,D5="Novembro","11",D5="Dezembro","12"))</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="7" spans="2:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="B7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="6"/>
-    </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
-        <v>0</v>
-      </c>
-      <c r="E11" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
-        <v>26</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B13" t="s">
-        <v>25</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="E14" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="E15" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="E16" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E17" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E18" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E19" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E20" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E21" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="22" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E22" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="23" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E23" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="24" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E24" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="25" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E25" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="26" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E26" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="27" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E27" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="28" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E28" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="29" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E29" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="30" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E30" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="31" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E31" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="32" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E32" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="33" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E33" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="34" spans="5:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="5:5">
       <c r="E34" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="35" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="36" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="49" x14ac:dyDescent="0.25"/>
-    <row r="50" x14ac:dyDescent="0.25"/>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="35" spans="5:5"/>
+    <row r="36" spans="5:5"/>
+    <row r="37" spans="5:5"/>
+    <row r="38" spans="5:5"/>
+    <row r="39" spans="5:5"/>
+    <row r="40" spans="5:5"/>
+    <row r="41" spans="5:5"/>
+    <row r="42" spans="5:5"/>
+    <row r="43" spans="5:5"/>
+    <row r="44" spans="5:5"/>
+    <row r="45" spans="5:5"/>
+    <row r="46" spans="5:5"/>
+    <row r="47" spans="5:5"/>
+    <row r="48" spans="5:5"/>
+    <row r="49"/>
+    <row r="50"/>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="1TE4otWnNaA/ODa3mDXOsTxBzUa7TNT/AWUKvPa+zIWelklZrAVOaRF2F/NV51e8NeLMZn5P9FQiQvWlZwWxMg==" saltValue="9pqYckD2lbbTQB2kN1v57A==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <protectedRanges>
@@ -841,7 +852,7 @@
   </protectedRanges>
   <dataConsolidate/>
   <conditionalFormatting sqref="D3 C5:D5 D7">
-    <cfRule type="containsBlanks" dxfId="0" priority="1">
+    <cfRule type="containsBlanks" dxfId="2" priority="1">
       <formula>LEN(TRIM(C3))=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -869,17 +880,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5a5f483f-f768-438e-b4ef-63f46a7558dd">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -888,7 +888,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006C56FB2846673243A9735D5EC6051572" ma:contentTypeVersion="11" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="36569ac63cfce8ff0f8884bc80e67f1c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5a5f483f-f768-438e-b4ef-63f46a7558dd" xmlns:ns3="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2040da04b75a9ea4fe796fa8180f8ca6" ns2:_="" ns3:_="">
     <xsd:import namespace="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
@@ -1083,40 +1083,25 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5a5f483f-f768-438e-b4ef-63f46a7558dd">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{637A4E3A-2793-49F4-B2B5-E8D79756ECAC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
-    <ds:schemaRef ds:uri="dd8c73df-45bd-468c-aae5-f3faedcbd5e2"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{380F78C4-C2DB-4920-B426-698322055391}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{380F78C4-C2DB-4920-B426-698322055391}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E5D4FB3-33A8-4BDC-8357-D4F39476A52A}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E5D4FB3-33A8-4BDC-8357-D4F39476A52A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
-    <ds:schemaRef ds:uri="dd8c73df-45bd-468c-aae5-f3faedcbd5e2"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{637A4E3A-2793-49F4-B2B5-E8D79756ECAC}"/>
 </file>
</xml_diff>

<commit_message>
Refactor functions for improved error handling and data extraction; update variable names for clarity; enhance PDF reading process with validation checks; add dynamic contract retrieval function.
</commit_message>
<xml_diff>
--- a/templates/Nomeador de arquivos.xlsx
+++ b/templates/Nomeador de arquivos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29101"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29122"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://incorporadoraampla.sharepoint.com/sites/Controladoria/Documentos Compartilhados/amplaGitHub/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="211" documentId="11_8BDB85793461764BD106A2AB1F101464FD041DB6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E1B558C-7DB6-4C72-878C-BA66BE5A1C3F}"/>
+  <xr:revisionPtr revIDLastSave="215" documentId="11_8BDB85793461764BD106A2AB1F101464FD041DB6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C013409-F692-569E-81BE-87543C994589}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1305" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -880,12 +880,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5a5f483f-f768-438e-b4ef-63f46a7558dd">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1084,18 +1086,16 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5a5f483f-f768-438e-b4ef-63f46a7558dd">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{380F78C4-C2DB-4920-B426-698322055391}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{637A4E3A-2793-49F4-B2B5-E8D79756ECAC}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1103,5 +1103,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{637A4E3A-2793-49F4-B2B5-E8D79756ECAC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{380F78C4-C2DB-4920-B426-698322055391}"/>
 </file>
</xml_diff>

<commit_message>
Add support for xcef8 file type in CEF processing functions; update NAMESPACE and documentation for e_abc_xabcs and e_cef_xcefs functions.
</commit_message>
<xml_diff>
--- a/templates/Nomeador de arquivos.xlsx
+++ b/templates/Nomeador de arquivos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29122"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29130"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://incorporadoraampla.sharepoint.com/sites/Controladoria/Documentos Compartilhados/amplaGitHub/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="215" documentId="11_8BDB85793461764BD106A2AB1F101464FD041DB6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C013409-F692-569E-81BE-87543C994589}"/>
+  <xr:revisionPtr revIDLastSave="217" documentId="11_8BDB85793461764BD106A2AB1F101464FD041DB6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8CD1A092-6F71-4555-9666-7301C613E44D}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1305" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -880,17 +880,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5a5f483f-f768-438e-b4ef-63f46a7558dd">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006C56FB2846673243A9735D5EC6051572" ma:contentTypeVersion="11" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="36569ac63cfce8ff0f8884bc80e67f1c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5a5f483f-f768-438e-b4ef-63f46a7558dd" xmlns:ns3="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2040da04b75a9ea4fe796fa8180f8ca6" ns2:_="" ns3:_="">
     <xsd:import namespace="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
@@ -1085,6 +1074,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5a5f483f-f768-438e-b4ef-63f46a7558dd">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1095,11 +1095,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E5D4FB3-33A8-4BDC-8357-D4F39476A52A}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{637A4E3A-2793-49F4-B2B5-E8D79756ECAC}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E5D4FB3-33A8-4BDC-8357-D4F39476A52A}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
feat: Update r_fechamento and r_xcef functions for improved data aggregation and filtering; modify Excel templates
</commit_message>
<xml_diff>
--- a/templates/Nomeador de arquivos.xlsx
+++ b/templates/Nomeador de arquivos.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="217" documentId="11_8BDB85793461764BD106A2AB1F101464FD041DB6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8CD1A092-6F71-4555-9666-7301C613E44D}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-1305" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nomeador" sheetId="1" r:id="rId1"/>
@@ -141,7 +141,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -275,17 +275,17 @@
   </cellStyles>
   <dxfs count="3">
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -365,9 +365,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0B4EABC4-6A33-4718-9BCE-E1A3BA547DAE}" name="empreendimentos" displayName="empreendimentos" ref="E11:E34" totalsRowShown="0" dataDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0B4EABC4-6A33-4718-9BCE-E1A3BA547DAE}" name="empreendimentos" displayName="empreendimentos" ref="E11:E34" totalsRowShown="0" dataDxfId="2">
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{9FD3D6E2-4108-48F3-8813-131FF4BB2FC6}" name="Empreendimentos" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{9FD3D6E2-4108-48F3-8813-131FF4BB2FC6}" name="Empreendimentos" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -637,7 +637,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J50"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" zeroHeight="1"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" zeroHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.7109375" customWidth="1"/>
     <col min="2" max="2" width="64.85546875" bestFit="1" customWidth="1"/>
@@ -652,13 +652,13 @@
     <col min="11" max="16384" width="9.140625" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6">
+    <row r="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B1" s="7" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="2:6"/>
-    <row r="3" spans="2:6" ht="21">
+    <row r="2" spans="2:6" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="2:6" ht="21" x14ac:dyDescent="0.35">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
@@ -667,8 +667,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="2:6"/>
-    <row r="5" spans="2:6" ht="21">
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="2:6" ht="21" x14ac:dyDescent="0.35">
       <c r="B5" s="5" t="s">
         <v>3</v>
       </c>
@@ -682,13 +682,13 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:6">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="F6" s="2" t="str">
         <f>_xlfn.CONCAT(IF(D3="Contratos (contr)","Contratos",IF(D3="Inadimplencia (inad)","Inadimplencia","")),"-",D7,"-",C5,"_",_xlfn.IFS(D5="Janeiro","01",D5="Fevereiro","02",D5="Março","03",D5="Abril","04",D5="Maio","05",D5="Junho","06",D5="Julho","07",D5="Agosto","08",D5="Setembro","09",D5="Outubro",10,D5="Novembro","11",D5="Dezembro","12"))</f>
         <v>Contratos-BUT-2025_07</v>
       </c>
     </row>
-    <row r="7" spans="2:6" ht="21">
+    <row r="7" spans="2:6" ht="21" x14ac:dyDescent="0.35">
       <c r="B7" s="5" t="s">
         <v>6</v>
       </c>
@@ -697,10 +697,10 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="2:6"/>
-    <row r="9" spans="2:6"/>
-    <row r="10" spans="2:6"/>
-    <row r="11" spans="2:6">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>8</v>
       </c>
@@ -708,7 +708,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="2:6">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>2</v>
       </c>
@@ -716,7 +716,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="2:6">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>11</v>
       </c>
@@ -724,127 +724,127 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="2:6">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E14" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="2:6">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E15" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="2:6">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E16" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="5:5">
+    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E17" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="5:5">
+    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E18" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="5:5">
+    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E19" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="5:5">
+    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E20" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="5:5">
+    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E21" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="5:5">
+    <row r="22" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E22" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="5:5">
+    <row r="23" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E23" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="5:5">
+    <row r="24" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E24" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="5:5">
+    <row r="25" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E25" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="5:5">
+    <row r="26" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E26" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="5:5">
+    <row r="27" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E27" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="5:5">
+    <row r="28" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E28" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="5:5">
+    <row r="29" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E29" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="5:5">
+    <row r="30" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E30" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="31" spans="5:5">
+    <row r="31" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E31" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="5:5">
+    <row r="32" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E32" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="33" spans="5:5">
+    <row r="33" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E33" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="34" spans="5:5">
+    <row r="34" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E34" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="35" spans="5:5"/>
-    <row r="36" spans="5:5"/>
-    <row r="37" spans="5:5"/>
-    <row r="38" spans="5:5"/>
-    <row r="39" spans="5:5"/>
-    <row r="40" spans="5:5"/>
-    <row r="41" spans="5:5"/>
-    <row r="42" spans="5:5"/>
-    <row r="43" spans="5:5"/>
-    <row r="44" spans="5:5"/>
-    <row r="45" spans="5:5"/>
-    <row r="46" spans="5:5"/>
-    <row r="47" spans="5:5"/>
-    <row r="48" spans="5:5"/>
-    <row r="49"/>
-    <row r="50"/>
+    <row r="35" spans="5:5" x14ac:dyDescent="0.25"/>
+    <row r="36" spans="5:5" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="5:5" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="5:5" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="5:5" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="5:5" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="5:5" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="5:5" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="5:5" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="5:5" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="5:5" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="5:5" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="5:5" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="5:5" x14ac:dyDescent="0.25"/>
+    <row r="49" x14ac:dyDescent="0.25"/>
+    <row r="50" x14ac:dyDescent="0.25"/>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="1TE4otWnNaA/ODa3mDXOsTxBzUa7TNT/AWUKvPa+zIWelklZrAVOaRF2F/NV51e8NeLMZn5P9FQiQvWlZwWxMg==" saltValue="9pqYckD2lbbTQB2kN1v57A==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <protectedRanges>
@@ -852,11 +852,11 @@
   </protectedRanges>
   <dataConsolidate/>
   <conditionalFormatting sqref="D3 C5:D5 D7">
-    <cfRule type="containsBlanks" dxfId="2" priority="1">
+    <cfRule type="containsBlanks" dxfId="0" priority="1">
       <formula>LEN(TRIM(C3))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <dataValidations disablePrompts="1" count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3" xr:uid="{6DF6D08E-F022-470A-82EF-7926C5CC47C9}">
       <formula1>INDIRECT("tipos[Tipos de arquivo]")</formula1>
     </dataValidation>
@@ -880,8 +880,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006C56FB2846673243A9735D5EC6051572" ma:contentTypeVersion="11" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="36569ac63cfce8ff0f8884bc80e67f1c">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5a5f483f-f768-438e-b4ef-63f46a7558dd" xmlns:ns3="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2040da04b75a9ea4fe796fa8180f8ca6" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006C56FB2846673243A9735D5EC6051572" ma:contentTypeVersion="11" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="ef780deaa56d3ced3ee4190a6bae4695">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5a5f483f-f768-438e-b4ef-63f46a7558dd" xmlns:ns3="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="468514e15a3503b4be0e7b051cba99cf" ns2:_="" ns3:_="">
     <xsd:import namespace="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
     <xsd:import namespace="dd8c73df-45bd-468c-aae5-f3faedcbd5e2"/>
     <xsd:element name="properties">
@@ -1075,6 +1075,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="5a5f483f-f768-438e-b4ef-63f46a7558dd">
@@ -1085,23 +1094,25 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E5D4FB3-33A8-4BDC-8357-D4F39476A52A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D05CCB86-8CE1-4FF5-83D3-4319A54535CC}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{637A4E3A-2793-49F4-B2B5-E8D79756ECAC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{380F78C4-C2DB-4920-B426-698322055391}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{380F78C4-C2DB-4920-B426-698322055391}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{637A4E3A-2793-49F4-B2B5-E8D79756ECAC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
+    <ds:schemaRef ds:uri="dd8c73df-45bd-468c-aae5-f3faedcbd5e2"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>